<commit_message>
updated the trip-list / new trip page
</commit_message>
<xml_diff>
--- a/KlimaChallenge_PM_v4.xlsx
+++ b/KlimaChallenge_PM_v4.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="59">
+  <fonts count="60">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -423,8 +423,14 @@
       <color rgb="00F59E0B"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00E95B20"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="26">
+  <fills count="27">
     <fill>
       <patternFill/>
     </fill>
@@ -568,6 +574,11 @@
         <fgColor rgb="00D6EEF5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="8">
     <border>
@@ -676,7 +687,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="496">
+  <cellXfs count="515">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2158,6 +2169,63 @@
     </xf>
     <xf numFmtId="0" fontId="55" fillId="21" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="21" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="21" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2413,7 +2481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="214" min="1" max="1"/>
@@ -2485,33 +2553,33 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" s="215">
-      <c r="A6" s="489" t="inlineStr">
+      <c r="A6" s="496" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B6" s="454" t="n"/>
+      <c r="C6" s="497" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D6" s="454" t="n"/>
+      <c r="E6" s="498" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B6" s="454" t="n"/>
-      <c r="C6" s="490" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="D6" s="454" t="n"/>
-      <c r="E6" s="491" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
       <c r="F6" s="454" t="n"/>
-      <c r="G6" s="492" t="inlineStr">
+      <c r="G6" s="499" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="H6" s="454" t="n"/>
-      <c r="I6" s="493" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="I6" s="500" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
       <c r="J6" s="454" t="n"/>
@@ -2519,7 +2587,7 @@
     <row r="7" ht="15.75" customHeight="1" s="215">
       <c r="A7" s="230" t="inlineStr">
         <is>
-          <t>prev sessions: 13 / 38 / 15 / 0 / 3   · Open Backlog = open feature/bug items; Pre-Prod Blockers = separate infra items not counted above</t>
+          <t>prev sessions: 13 / 39 / 14 / 0 / 3   · Open Backlog = open feature/bug items; Pre-Prod Blockers = separate infra items not counted above</t>
         </is>
       </c>
       <c r="B7" s="459" t="n"/>
@@ -3281,6 +3349,39 @@
       <c r="G34" s="265" t="inlineStr">
         <is>
           <t>██░░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="215">
+      <c r="A35" s="501" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B35" s="502" t="inlineStr">
+        <is>
+          <t>Mar 16</t>
+        </is>
+      </c>
+      <c r="C35" s="503" t="inlineStr">
+        <is>
+          <t>DateTimePicker + full Trips screen + profile nav rework</t>
+        </is>
+      </c>
+      <c r="D35" s="504" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" s="505" t="inlineStr">
+        <is>
+          <t>Feature / UX</t>
+        </is>
+      </c>
+      <c r="F35" s="506" t="n">
+        <v>53</v>
+      </c>
+      <c r="G35" s="507" t="inlineStr">
+        <is>
+          <t>███░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -3318,7 +3419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="214" min="1" max="1"/>
@@ -4176,8 +4277,70 @@
       <c r="K17" s="459" t="n"/>
       <c r="L17" s="454" t="n"/>
     </row>
-    <row r="18">
-      <c r="A18" s="304" t="inlineStr">
+    <row r="18" ht="90" customHeight="1" s="215">
+      <c r="A18" s="292" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B18" s="293" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C18" s="294" t="inlineStr">
+        <is>
+          <t>Native DateTimePicker · Trips list screen · Profile layout rework</t>
+        </is>
+      </c>
+      <c r="D18" s="295" t="inlineStr">
+        <is>
+          <t>#42 DateTimePicker: replaced custom 7-day date scroll + manual HH:MM inputs with @react-native-community/datetimepicker in both QuickAddTripModal and TripDetailModal. iOS: spinner display inline + Done button. Android: system dialog. Single Date state (no hour/minute strings). Plugin added to app.config.ts. Requires custom dev build (not Expo Go). Recent Trips rework: main screen now groups preview trips by date (date group headers). New app/trips.tsx screen: filter chips (All/Bus/Train/Tram/Subway), full date-grouped list, swipe-left-to-delete (RNGH Pan, -80px threshold, red zone, 200ms fly-off). 'See all X trips' navigates to /trips. New utils/tripGrouping.ts shared helper (formatDateLabel, groupTripsByDate). Deleted dead stubs app/new-trip.tsx + app/trip/[id].tsx. Profile rework: new layout order — Avatar → Display Name + KlimaTicket + Save → navSection (Stats / Achievements / My Trips) → Danger Zone. My Trips button added (MaterialIcons format-list-bulleted, routes to /trips). Files: app.config.ts, components/ui/QuickAddTripModal.tsx, components/ui/TripDetailModal.tsx, app/(tabs)/user.tsx, app/(tabs)/_user_styles.tsx, app/trips.tsx (new), app/profile.tsx, utils/tripGrouping.ts (new)</t>
+        </is>
+      </c>
+      <c r="E18" s="296" t="inlineStr">
+        <is>
+          <t>DateTimePicker: users had no way to backfill past trips — critical real-world usage gap. Trips screen: inline 'show all' expansion had no filter/delete; a dedicated screen matches the mental model of a full trip history. Profile rework: display name + KlimaTicket were buried below nav shortcuts; moving them above improves discoverability and data-entry flow.</t>
+        </is>
+      </c>
+      <c r="F18" s="297" t="inlineStr">
+        <is>
+          <t>CRLF + 4-tab indentation in user.tsx and profile.tsx caused Edit tool to repeatedly fail string matching. Diagnosed with cat -A, resolved by writing complete file rewrites. Typo in user.tsx Write (missing } in JSX) caused cascade of TS parse errors — fixed with targeted edit. theme='dark' prop removal from TripRouteFields caused TS error (prop removed in S11 tech debt).</t>
+        </is>
+      </c>
+      <c r="G18" s="298" t="inlineStr">
+        <is>
+          <t>DateTimePicker: expo-datetime-picker considered but requires native module build anyway; @react-native-community/datetimepicker chosen as more stable and widely used. Trips screen: ScrollView-based swipe vs RNGH Pan — RNGH chosen for correct gesture priority negotiation with parent ScrollView (activeOffsetX + failOffsetY).</t>
+        </is>
+      </c>
+      <c r="H18" s="299" t="inlineStr">
+        <is>
+          <t>DateTimePicker requires custom dev build — document in project state. Swipe card needs opaque backgroundColor (blue.dark) to hide semi-transparent card bleed over red delete zone. Cross-screen sync: trips.tsx writes directly to AsyncStorage; user.tsx picks up via useFocusEffect (no shared state needed). CRLF files must be fully rewritten — Edit tool cannot reliably match Windows line endings.</t>
+        </is>
+      </c>
+      <c r="I18" s="300" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J18" s="301" t="inlineStr">
+        <is>
+          <t>~5h</t>
+        </is>
+      </c>
+      <c r="K18" s="302" t="inlineStr">
+        <is>
+          <t>UX Design / Interaction Design</t>
+        </is>
+      </c>
+      <c r="L18" s="303" t="inlineStr">
+        <is>
+          <t>[To be completed via web interface]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="304" t="inlineStr">
         <is>
           <t>Column colour guide:  E (green) = Why / rationale  ·  F (red) = Problems  ·  H (blue) = Standing decisions  ·  L (purple) = Retrospective reflection</t>
         </is>
@@ -4880,7 +5043,7 @@
       </c>
       <c r="I6" s="347" t="inlineStr">
         <is>
-          <t>Add AsyncStorage.multiRemove for all 4 keys in handleDeleteAllTrips in profile.tsx  ·  Completed S13 — AsyncStorage.multiRemove(['@claimedQuests','@claimedAchievements','@dailyQuestSelection','@weeklyQuestSelection']) in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips</t>
+          <t>Add AsyncStorage.multiRemove for all 4 keys in handleDeleteAllTrips in profile.tsx  ·  Completed S13 — AsyncStorage.multiRemove(['@claimedQuests','@claimedAchievements','@dailyQuestSelection','@weeklyQuestSelection']) in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips</t>
         </is>
       </c>
     </row>
@@ -4927,7 +5090,7 @@
       </c>
       <c r="I7" s="347" t="inlineStr">
         <is>
-          <t>Change fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts</t>
+          <t>Change fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts</t>
         </is>
       </c>
     </row>
@@ -4974,7 +5137,7 @@
       </c>
       <c r="I8" s="347" t="inlineStr">
         <is>
-          <t>TouchableWithoutFeedback wrapper or onStartShouldSetResponder pattern  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown sits at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown sits at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown at zIndex 11</t>
+          <t>TouchableWithoutFeedback wrapper or onStartShouldSetResponder pattern  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown sits at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown sits at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown at zIndex 11</t>
         </is>
       </c>
     </row>
@@ -5210,54 +5373,54 @@
       </c>
       <c r="I14" s="347" t="inlineStr">
         <is>
-          <t>Stats: replace chart with illustration + CTA. Quests: show locked state with Add a trip to start earning XP prompt.  ·  Completed S13 — Stats: full empty state replacing data sections. Quests: info banner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="48" customHeight="1" s="215">
-      <c r="A15" s="469" t="inlineStr">
+          <t>Stats: replace chart with illustration + CTA. Quests: show locked state with Add a trip to start earning XP prompt.  ·  Completed S13 — Stats: full empty state replacing data sections. Quests: info banner.  ·  Completed S13 — Stats: full empty state replacing data sections. Quests: info banner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1" s="215">
+      <c r="A15" s="508" t="inlineStr">
         <is>
           <t>42</t>
         </is>
       </c>
-      <c r="B15" s="470" t="inlineStr">
+      <c r="B15" s="509" t="inlineStr">
         <is>
           <t>UX</t>
         </is>
       </c>
-      <c r="C15" s="469" t="inlineStr">
+      <c r="C15" s="508" t="inlineStr">
         <is>
           <t>Manual date/time for trips</t>
         </is>
       </c>
-      <c r="D15" s="470" t="inlineStr">
+      <c r="D15" s="509" t="inlineStr">
         <is>
           <t>Users can only log trips at the current moment. No way to backfill yesterday's commute. A date/time picker on the Add Trip modal is needed for real-world usage.</t>
         </is>
       </c>
-      <c r="E15" s="471" t="inlineStr">
+      <c r="E15" s="509" t="inlineStr">
         <is>
           <t>🟠 High</t>
         </is>
       </c>
-      <c r="F15" s="470" t="inlineStr">
+      <c r="F15" s="509" t="inlineStr">
         <is>
           <t>S (2-4h)</t>
         </is>
       </c>
-      <c r="G15" s="470" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H15" s="470" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="I15" s="472" t="inlineStr">
-        <is>
-          <t>Add DateTimePicker (expo-datetime-picker or RN DateTimePicker) to QuickAddTripModal. Default to now, allow past dates.</t>
+      <c r="G15" s="345" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H15" s="346" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="I15" s="347" t="inlineStr">
+        <is>
+          <t>Add DateTimePicker (expo-datetime-picker or RN DateTimePicker) to QuickAddTripModal. Default to now, allow past dates.  ·  Completed S14 — Native DateTimePicker in both modals; iOS spinner+Done, Android dialog; single Date state</t>
         </is>
       </c>
     </row>
@@ -7130,7 +7293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="214" min="1" max="1"/>
@@ -7673,6 +7836,43 @@
       <c r="G17" s="374" t="inlineStr">
         <is>
           <t>Academic rigour / Data sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="56" customHeight="1" s="215">
+      <c r="A18" s="510" t="inlineStr">
+        <is>
+          <t>CRLF files + Edit tool string matching</t>
+        </is>
+      </c>
+      <c r="B18" s="469" t="inlineStr">
+        <is>
+          <t>Files with Windows CRLF line endings must be fully rewritten — never use targeted Edit.</t>
+        </is>
+      </c>
+      <c r="C18" s="470" t="inlineStr">
+        <is>
+          <t>The Edit tool matches exact byte strings. CRLF (\r\n) line endings cause every match to fail silently or partially, leading to cascading TS errors or phantom rewrites. Diagnosed via cat -A; the only reliable fix is a full Write of the affected file.</t>
+        </is>
+      </c>
+      <c r="D18" s="511" t="inlineStr">
+        <is>
+          <t>Edit silently fails, file unchanged; downstream TS errors if a partial write occurs.</t>
+        </is>
+      </c>
+      <c r="E18" s="512" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="F18" s="513" t="inlineStr">
+        <is>
+          <t>🟠 High</t>
+        </is>
+      </c>
+      <c r="G18" s="514" t="inlineStr">
+        <is>
+          <t>Platform limitations / DX</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S15/S16 added streak mechanics and haptic feedback, log-again for trips.
</commit_message>
<xml_diff>
--- a/KlimaChallenge_PM_v4.xlsx
+++ b/KlimaChallenge_PM_v4.xlsx
@@ -687,7 +687,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="515">
+  <cellXfs count="544">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2226,6 +2226,93 @@
     </xf>
     <xf numFmtId="0" fontId="51" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="26" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2481,7 +2568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="214" min="1" max="1"/>
@@ -2553,31 +2640,31 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" s="215">
-      <c r="A6" s="496" t="inlineStr">
-        <is>
-          <t>14</t>
+      <c r="A6" s="515" t="inlineStr">
+        <is>
+          <t>16</t>
         </is>
       </c>
       <c r="B6" s="454" t="n"/>
-      <c r="C6" s="497" t="inlineStr">
-        <is>
-          <t>42</t>
+      <c r="C6" s="516" t="inlineStr">
+        <is>
+          <t>46</t>
         </is>
       </c>
       <c r="D6" s="454" t="n"/>
-      <c r="E6" s="498" t="inlineStr">
-        <is>
-          <t>13</t>
+      <c r="E6" s="517" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="F6" s="454" t="n"/>
-      <c r="G6" s="499" t="inlineStr">
+      <c r="G6" s="518" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="H6" s="454" t="n"/>
-      <c r="I6" s="500" t="inlineStr">
+      <c r="I6" s="519" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -2587,7 +2674,7 @@
     <row r="7" ht="15.75" customHeight="1" s="215">
       <c r="A7" s="230" t="inlineStr">
         <is>
-          <t>prev sessions: 13 / 39 / 14 / 0 / 3   · Open Backlog = open feature/bug items; Pre-Prod Blockers = separate infra items not counted above</t>
+          <t>prev sessions: 15 / 44 / 11 / 0 / 5   · Open Backlog = open feature/bug items; Pre-Prod Blockers = separate infra items not counted above</t>
         </is>
       </c>
       <c r="B7" s="459" t="n"/>
@@ -3382,6 +3469,72 @@
       <c r="G35" s="507" t="inlineStr">
         <is>
           <t>███░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="215">
+      <c r="A36" s="520" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B36" s="521" t="inlineStr">
+        <is>
+          <t>Mar 16</t>
+        </is>
+      </c>
+      <c r="C36" s="261" t="inlineStr">
+        <is>
+          <t>Haptic feedback throughout + streak system + streak badge on level card</t>
+        </is>
+      </c>
+      <c r="D36" s="522" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="523" t="inlineStr">
+        <is>
+          <t>Gamification / Polish</t>
+        </is>
+      </c>
+      <c r="F36" s="524" t="n">
+        <v>55</v>
+      </c>
+      <c r="G36" s="525" t="inlineStr">
+        <is>
+          <t>██░░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="215">
+      <c r="A37" s="526" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B37" s="527" t="inlineStr">
+        <is>
+          <t>Mar 16</t>
+        </is>
+      </c>
+      <c r="C37" s="503" t="inlineStr">
+        <is>
+          <t>Streak milestone XP rewards + Log Again (replaces #47 recurring trip)</t>
+        </is>
+      </c>
+      <c r="D37" s="528" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="529" t="inlineStr">
+        <is>
+          <t>Gamification / UX</t>
+        </is>
+      </c>
+      <c r="F37" s="530" t="n">
+        <v>57</v>
+      </c>
+      <c r="G37" s="531" t="inlineStr">
+        <is>
+          <t>██░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="214" min="1" max="1"/>
@@ -4339,8 +4492,132 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="304" t="inlineStr">
+    <row r="19" ht="90" customHeight="1" s="215">
+      <c r="A19" s="532" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B19" s="533" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C19" s="534" t="inlineStr">
+        <is>
+          <t>Haptic feedback · Streak system · UserLevelCard streak badge</t>
+        </is>
+      </c>
+      <c r="D19" s="535" t="inlineStr">
+        <is>
+          <t>#45 Haptic feedback: expo-haptics wired throughout the app. ImpactFeedbackStyle.Medium on trip add (QuickAdd) and swipe-delete in trips.tsx. ImpactFeedbackStyle.Light on favorite card long-press add. NotificationFeedbackType.Success on level-up, quest/achievement/main-quest claim. #43 Streak system: new utils/streakSystem.ts with computeStreak(trips) — counts consecutive calendar days ending today or yesterday, returns 0 if streak broken. Displayed in UserLevelCard footer as 🔥 Xd badge (Palette.red.light, MaterialIcons local-fire-department). streak computed via useMemo([trips]) in user.tsx and passed as prop. Hidden when streak = 0. Files: utils/streakSystem.ts (new), components/ui/UserLevelCard.tsx, app/(tabs)/user.tsx (Write), app/trips.tsx, app/quests.tsx</t>
+        </is>
+      </c>
+      <c r="E19" s="536" t="inlineStr">
+        <is>
+          <t>Haptics are table-stakes polish for a native app — they make every interaction feel intentional. Streak is a core retention mechanic; showing it on the level card keeps it visible without requiring a dedicated screen.</t>
+        </is>
+      </c>
+      <c r="F19" s="537" t="inlineStr">
+        <is>
+          <t>expo-haptics was already installed (expo SDK default) — no install needed. user.tsx required full Write (CRLF file).</t>
+        </is>
+      </c>
+      <c r="G19" s="538" t="inlineStr">
+        <is>
+          <t>Considered storing streak in AsyncStorage to avoid recomputing — rejected because computing from the trips array is O(n) and always accurate; no sync risk.</t>
+        </is>
+      </c>
+      <c r="H19" s="539" t="inlineStr">
+        <is>
+          <t>Streak starts from today if today has a trip, otherwise from yesterday — prevents streak breaking just because the user hasn't logged today's trip yet.</t>
+        </is>
+      </c>
+      <c r="I19" s="540" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J19" s="541" t="inlineStr">
+        <is>
+          <t>~2h</t>
+        </is>
+      </c>
+      <c r="K19" s="542" t="inlineStr">
+        <is>
+          <t>Gamification / Engagement</t>
+        </is>
+      </c>
+      <c r="L19" s="543" t="inlineStr">
+        <is>
+          <t>[To be completed via web interface]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1" s="215">
+      <c r="A20" s="532" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B20" s="533" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C20" s="534" t="inlineStr">
+        <is>
+          <t>Streak milestone rewards · Log Again button · QuickAdd prefill</t>
+        </is>
+      </c>
+      <c r="D20" s="535" t="inlineStr">
+        <is>
+          <t>Streak milestones: STREAK_MILESTONES array (3/7/14/30/60/100 days → 50/150/300/600/1000/2000 XP) and getNewMilestoneXP(streak, claimed) added to utils/streakSystem.ts. claimedMilestones state in user.tsx loaded on init/focus from @claimedStreakMilestones. After each trip add, checkStreakMilestones fires; if a milestone is newly hit, bonus XP awarded 1.8s after trip toast (haptic + level-up if triggered). Log Again: onLogAgain prop added to TripDetailModal; view mode shows Close + Log Again two-button row (green, replay icon). QuickAddTripModal gains optional prefill prop (PrefillData type) with useEffect([visible]) that populates all fields when modal opens; date resets to now. handleLogAgain in user.tsx: closes detail modal → sets prefillData state → opens QuickAdd. Files: utils/streakSystem.ts, components/ui/TripDetailModal.tsx, components/ui/QuickAddTripModal.tsx, app/(tabs)/user.tsx (Write)</t>
+        </is>
+      </c>
+      <c r="E20" s="536" t="inlineStr">
+        <is>
+          <t>Milestone rewards give the streak system progression depth beyond a simple counter — they reward users who maintain long streaks and make the streak feel meaningful. Log Again replaces the vague #47 'recurring trip' item: favorites already handle the high-frequency repeat case; Log Again fills the gap for any past trip regardless of frequency.</t>
+        </is>
+      </c>
+      <c r="F20" s="537" t="inlineStr">
+        <is>
+          <t>TripDetailModal Edit tool failed on first attempt (indentation mismatch); resolved by re-reading exact whitespace before editing. Milestone XP toast coordination: two toasts in quick succession (trip XP + milestone XP) resolved by delaying milestone toast by 1.8s.</t>
+        </is>
+      </c>
+      <c r="G20" s="538" t="inlineStr">
+        <is>
+          <t>Milestone XP could be summed with trip XP and shown in one toast — rejected because the delay makes the milestone feel like a separate reward rather than noise. Log Again could have re-logged without opening QuickAdd — rejected because user should be able to adjust the date/time before confirming.</t>
+        </is>
+      </c>
+      <c r="H20" s="539" t="inlineStr">
+        <is>
+          <t>Milestone awards are one-time (persisted to @claimedStreakMilestones) — a streak breaking and restarting does NOT re-award. prefill date always resets to now (not the original trip date) — the intent is to log a new trip today, not to duplicate a past date.</t>
+        </is>
+      </c>
+      <c r="I20" s="540" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J20" s="541" t="inlineStr">
+        <is>
+          <t>~3h</t>
+        </is>
+      </c>
+      <c r="K20" s="542" t="inlineStr">
+        <is>
+          <t>Gamification / Engagement</t>
+        </is>
+      </c>
+      <c r="L20" s="543" t="inlineStr">
+        <is>
+          <t>[To be completed via web interface]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="304" t="inlineStr">
         <is>
           <t>Column colour guide:  E (green) = Why / rationale  ·  F (red) = Problems  ·  H (blue) = Standing decisions  ·  L (purple) = Retrospective reflection</t>
         </is>
@@ -5043,7 +5320,7 @@
       </c>
       <c r="I6" s="347" t="inlineStr">
         <is>
-          <t>Add AsyncStorage.multiRemove for all 4 keys in handleDeleteAllTrips in profile.tsx  ·  Completed S13 — AsyncStorage.multiRemove(['@claimedQuests','@claimedAchievements','@dailyQuestSelection','@weeklyQuestSelection']) in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips</t>
+          <t>Add AsyncStorage.multiRemove for all 4 keys in handleDeleteAllTrips in profile.tsx  ·  Completed S13 — AsyncStorage.multiRemove(['@claimedQuests','@claimedAchievements','@dailyQuestSelection','@weeklyQuestSelection']) in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips  ·  Completed S13 — AsyncStorage.multiRemove for all 4 quest/achievement keys in handleDeleteAllTrips</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5367,7 @@
       </c>
       <c r="I7" s="347" t="inlineStr">
         <is>
-          <t>Change fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts</t>
+          <t>Change fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts  ·  Completed S13 — Changed fallback from `return initialTrips` to `return []` in tripStorage.ts</t>
         </is>
       </c>
     </row>
@@ -5137,7 +5414,7 @@
       </c>
       <c r="I8" s="347" t="inlineStr">
         <is>
-          <t>TouchableWithoutFeedback wrapper or onStartShouldSetResponder pattern  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown sits at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown sits at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown at zIndex 11</t>
+          <t>TouchableWithoutFeedback wrapper or onStartShouldSetResponder pattern  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown sits at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown sits at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown at zIndex 11  ·  Completed S13 — Absolute TouchableWithoutFeedback overlay (zIndex 10) closes dropdown; dropdown at zIndex 11</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5650,7 @@
       </c>
       <c r="I14" s="347" t="inlineStr">
         <is>
-          <t>Stats: replace chart with illustration + CTA. Quests: show locked state with Add a trip to start earning XP prompt.  ·  Completed S13 — Stats: full empty state replacing data sections. Quests: info banner.  ·  Completed S13 — Stats: full empty state replacing data sections. Quests: info banner.</t>
+          <t>Stats: replace chart with illustration + CTA. Quests: show locked state with Add a trip to start earning XP prompt.  ·  Completed S13 — Stats: full empty state replacing data sections. Quests: info banner.  ·  Completed S13 — Stats: full empty state replacing data sections. Quests: info banner.  ·  Completed S13 — Stats: full empty state replacing data sections. Quests: info banner.</t>
         </is>
       </c>
     </row>
@@ -5420,54 +5697,54 @@
       </c>
       <c r="I15" s="347" t="inlineStr">
         <is>
-          <t>Add DateTimePicker (expo-datetime-picker or RN DateTimePicker) to QuickAddTripModal. Default to now, allow past dates.  ·  Completed S14 — Native DateTimePicker in both modals; iOS spinner+Done, Android dialog; single Date state</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="48" customHeight="1" s="215">
-      <c r="A16" s="469" t="inlineStr">
+          <t>Add DateTimePicker (expo-datetime-picker or RN DateTimePicker) to QuickAddTripModal. Default to now, allow past dates.  ·  Completed S14 — Native DateTimePicker in both modals; iOS spinner+Done, Android dialog; single Date state  ·  Completed S14 — Native DateTimePicker in both modals; iOS spinner+Done, Android dialog; single Date state</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1" s="215">
+      <c r="A16" s="508" t="inlineStr">
         <is>
           <t>43</t>
         </is>
       </c>
-      <c r="B16" s="470" t="inlineStr">
+      <c r="B16" s="509" t="inlineStr">
         <is>
           <t>Gamification</t>
         </is>
       </c>
-      <c r="C16" s="469" t="inlineStr">
+      <c r="C16" s="508" t="inlineStr">
         <is>
           <t>Streak system</t>
         </is>
       </c>
-      <c r="D16" s="470" t="inlineStr">
+      <c r="D16" s="509" t="inlineStr">
         <is>
           <t>Track consecutive days the user logs at least one trip. Display streak on UserLevelCard. Streak loss is a powerful retention mechanic (loss aversion). Fits thesis well.</t>
         </is>
       </c>
-      <c r="E16" s="471" t="inlineStr">
+      <c r="E16" s="509" t="inlineStr">
         <is>
           <t>🟠 High</t>
         </is>
       </c>
-      <c r="F16" s="470" t="inlineStr">
+      <c r="F16" s="509" t="inlineStr">
         <is>
           <t>M (4-8h)</t>
         </is>
       </c>
-      <c r="G16" s="470" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H16" s="470" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="I16" s="472" t="inlineStr">
-        <is>
-          <t>AsyncStorage key @currentStreak + @lastTripDate. Streak breaks if no trip logged by midnight. Consider streak freeze item as future extension.</t>
+      <c r="G16" s="345" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H16" s="346" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="I16" s="347" t="inlineStr">
+        <is>
+          <t>AsyncStorage key @currentStreak + @lastTripDate. Streak breaks if no trip logged by midnight. Consider streak freeze item as future extension.  ·  Completed S15 — computeStreak utility + 🔥 badge on UserLevelCard</t>
         </is>
       </c>
     </row>
@@ -5518,50 +5795,50 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1" s="215">
-      <c r="A18" s="473" t="inlineStr">
+    <row r="18" ht="28" customHeight="1" s="215">
+      <c r="A18" s="508" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="B18" s="474" t="inlineStr">
+      <c r="B18" s="509" t="inlineStr">
         <is>
           <t>UX</t>
         </is>
       </c>
-      <c r="C18" s="473" t="inlineStr">
+      <c r="C18" s="508" t="inlineStr">
         <is>
           <t>Haptic feedback</t>
         </is>
       </c>
-      <c r="D18" s="474" t="inlineStr">
+      <c r="D18" s="509" t="inlineStr">
         <is>
           <t>Add haptic feedback on: trip add confirmation, XP toast, quest claim, level-up, slide-to-delete confirm. Quick win for perceived quality.</t>
         </is>
       </c>
-      <c r="E18" s="475" t="inlineStr">
+      <c r="E18" s="509" t="inlineStr">
         <is>
           <t>🟡 Medium</t>
         </is>
       </c>
-      <c r="F18" s="474" t="inlineStr">
+      <c r="F18" s="509" t="inlineStr">
         <is>
           <t>XS (1h)</t>
         </is>
       </c>
-      <c r="G18" s="474" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H18" s="474" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="I18" s="476" t="inlineStr">
-        <is>
-          <t>Use expo-haptics. Haptics.impactAsync(ImpactFeedbackStyle.Medium) for most; Heavy for level-up.</t>
+      <c r="G18" s="345" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H18" s="346" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="I18" s="347" t="inlineStr">
+        <is>
+          <t>Use expo-haptics. Haptics.impactAsync(ImpactFeedbackStyle.Medium) for most; Heavy for level-up.  ·  Completed S15 — expo-haptics wired to all key interactions</t>
         </is>
       </c>
     </row>
@@ -5612,50 +5889,50 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1" s="215">
-      <c r="A20" s="477" t="inlineStr">
+    <row r="20" ht="28" customHeight="1" s="215">
+      <c r="A20" s="508" t="inlineStr">
         <is>
           <t>47</t>
         </is>
       </c>
-      <c r="B20" s="478" t="inlineStr">
+      <c r="B20" s="509" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="C20" s="477" t="inlineStr">
+      <c r="C20" s="508" t="inlineStr">
         <is>
           <t>Recurring trip / one-tap repeat</t>
         </is>
       </c>
-      <c r="D20" s="478" t="inlineStr">
+      <c r="D20" s="509" t="inlineStr">
         <is>
           <t>Allow users to repeat a previous trip with one tap — pre-fills all fields from the last matching trip. Reduces friction for daily commuters.</t>
         </is>
       </c>
-      <c r="E20" s="479" t="inlineStr">
+      <c r="E20" s="509" t="inlineStr">
         <is>
           <t>🔵 Low</t>
         </is>
       </c>
-      <c r="F20" s="478" t="inlineStr">
+      <c r="F20" s="509" t="inlineStr">
         <is>
           <t>S (2-4h)</t>
         </is>
       </c>
-      <c r="G20" s="478" t="inlineStr">
-        <is>
-          <t>⬜ Todo</t>
-        </is>
-      </c>
-      <c r="H20" s="478" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="I20" s="480" t="inlineStr">
-        <is>
-          <t>Could surface as a 'Repeat' button in TripDetailModal or as a quick-action in the favorites section.</t>
+      <c r="G20" s="345" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="H20" s="346" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="I20" s="347" t="inlineStr">
+        <is>
+          <t>Could surface as a 'Repeat' button in TripDetailModal or as a quick-action in the favorites section.  ·  Completed S16 — Replaced by Log Again button in TripDetailModal + QuickAdd prefill prop</t>
         </is>
       </c>
     </row>

</xml_diff>